<commit_message>
feat(essay): integrate 775 model answers, rubrics, and Internet references across web UI and exports
</commit_message>
<xml_diff>
--- a/TONG_HOP_QUIZ_15_NGAY_EXCEL/02_FULL_NGAN_HANG_1679_CAU_CHI_TIET_CHIA_20_CAU/Day_01_Full_150_Cau/Day_01_Ngan_Hang_Phan_01_19_Cau.xlsx
+++ b/TONG_HOP_QUIZ_15_NGAY_EXCEL/02_FULL_NGAN_HANG_1679_CAU_CHI_TIET_CHIA_20_CAU/Day_01_Full_150_Cau/Day_01_Ngan_Hang_Phan_01_19_Cau.xlsx
@@ -884,10 +884,15 @@
       <c r="K8" s="3" t="inlineStr">
         <is>
           <t>👉 Tiêu chí chấm (Rubric 3 điểm):
-- Đúng bản chất vấn đề và yêu cầu kỹ thuật.
-- Đầy đủ các tiêu chí chấp nhận / test case tối thiểu.
-- Gợi ý cốt lõi: Với mỗi mũi tên, hỏi: phần việc nào đang do con người làm thủ công và phương pháp sau chuyển phần việc đó sang đâu?
-Phân tích theo nguyên lý thiết kế: Với mỗi mũi tên, hỏi: phần việc nào đang do con người làm thủ công và phương pháp sau chuyển phần việc đó sang đâu?</t>
+- Điểm nghẽn hệ chuyên gia (1.5 điểm): Nêu rõ nghẽn thu nhận tri thức (knowledge acquisition bottleneck), bùng nổ tổ hợp quy tắc mâu thuẫn/ngoại lệ và tính giòn (brittle) khi mở rộng.
+- Đóng góp của Deep Learning (1.5 điểm): Nêu rõ việc loại bỏ trích xuất đặc trưng thủ công (handcrafted feature engineering) và chuyển sang học biểu diễn tự động phân tầng (end-to-end representation learning).
+CÂU TRẢ LỜI MẪU CHI TIẾT:
+1. Điểm nghẽn của hệ chuyên gia (Expert Systems): Xảy ra hiện tượng 'nghẽn cổ chai thu nhận tri thức' (knowledge acquisition bottleneck). Tri thức chuyên gia trong thực tế mang tính ngầm định (tacit knowledge), mơ hồ và chứa vô số ngoại lệ. Việc viết và duy trì hàng ngàn quy tắc 'if-then' thủ công dẫn đến sự bùng nổ tổ hợp (combinatorial explosion), xung đột quy tắc và hệ thống trở nên cực kỳ giòn (brittle) — chỉ cần một dữ liệu ngoài dự liệu là hệ thống tê liệt hoàn toàn, không thể tự mở rộng.
+2. Phần việc thủ công mà Deep Learning đã giảm bớt so với Machine Learning thống kê: Deep Learning loại bỏ hoàn toàn khâu trích xuất và thiết kế đặc trưng thủ công (manual feature engineering / handcrafted features). Trong ML thống kê cổ điển, kỹ sư phải tự tay thiết kế các hàm trích xuất đặc trưng (như SIFT, HOG, n-gram). Deep Learning thay thế khâu này bằng kiến trúc mạng nơ-ron nhiều tầng có khả năng học biểu diễn đặc trưng phân tầng tự động (hierarchical representation learning / end-to-end) trực tiếp từ dữ liệu thô.
+PHÂN TÍCH THEO NGUYÊN LÝ THIẾT KẾ:
+Phân tích theo nguyên lý thiết kế: Sự tiến hóa từ hệ chuyên gia sang ML thống kê và Deep Learning phản ánh quy luật chuyển giao công việc từ con người sang thuật toán tính toán. Hệ chuyên gia yêu cầu con người tự viết cả quy tắc và logic; ML thống kê giải phóng con người khỏi việc viết luật suy diễn nhưng vẫn bắt con người thiết kế đặc trưng (features); Deep Learning với kiến trúc nơ-ron phân tầng giải quyết triệt để khâu biểu diễn (representation learning), tạo điều kiện cho các mô hình nền tảng (Foundation Models) mở rộng quy mô dữ liệu và tham số không giới hạn.
+NGUỒN THAM KHẢO &amp; TÀI LIỆU KỸ THUẬT:
+LeCun, Y., Bengio, Y., &amp; Hinton, G. (2015). Deep learning. Nature, 521(7553), 436-444. https://doi.org/10.1038/nature14539; Russell, S., &amp; Norvig, P. (2020). Artificial Intelligence: A Modern Approach (4th ed.). Pearson.</t>
         </is>
       </c>
     </row>
@@ -1127,10 +1132,17 @@
       <c r="K13" s="3" t="inlineStr">
         <is>
           <t>👉 Tiêu chí chấm (Rubric 3 điểm):
-- Đúng bản chất vấn đề và yêu cầu kỹ thuật.
-- Đầy đủ các tiêu chí chấp nhận / test case tối thiểu.
-- Gợi ý cốt lõi: Liệt kê tính năng đã có, rồi kiểm tra xem hệ thống có thể hành động và quan sát kết quả của hành động đó hay không.
-Phân tích theo nguyên lý thiết kế: Liệt kê tính năng đã có, rồi kiểm tra xem hệ thống có thể hành động và quan sát kết quả của hành động đó hay không.</t>
+- Phân loại vị trí trên trục (1.0 điểm): Xác định đúng hệ thống là Chatbot có RAG/Memory, nằm giữa LLM độc lập và Agent.
+- Hai tính năng vượt trội (1.0 điểm): Nêu chính xác truy xuất FAQ (RAG) và bộ nhớ ngữ cảnh 5 lượt gần nhất.
+- Năng lực còn thiếu cốt lõi (1.0 điểm): Nêu rõ khả năng tự chủ gọi công cụ (tool/function calling) và xử lý kết quả quan sát môi trường.
+CÂU TRẢ LỜI MẪU CHI TIẾT:
+- Xếp hệ thống trên trục: Hệ thống nằm ở mức 'Retrieval-Augmented Chatbot' (Chatbot có bộ nhớ và truy xuất ngữ cảnh), cao hơn LLM độc lập (standalone LLM) nhưng chưa đạt tới mức Agent tự chủ (Autonomous Tool-Using Agent).
+- Hai tính năng mạnh hơn LLM độc lập: (1) Khả năng grounded tri thức bên ngoài qua truy xuất câu hỏi thường gặp (FAQ RAG), giúp giảm thiểu ảo giác và cung cấp câu trả lời chính xác theo tài liệu nghiệp vụ; (2) Lưu giữ trạng thái ngữ cảnh hội thoại qua 5 lượt trao đổi gần nhất (short-term conversation memory), cho phép hiểu các câu hỏi nối tiếp và đại từ thay thế.
+- Một năng lực còn thiếu để trở thành agent dùng công cụ: Khả năng tự chủ gọi công cụ (Tool / Function Calling) và vòng lặp phản hồi ReAct (Action -&gt; Observation). Hiện tại hệ thống không thể tự quyết định khi nào cần gọi API bên ngoài, không thể truyền tham số có cấu trúc và không thể quan sát kết quả từ công cụ để suy luận tiếp.
+PHÂN TÍCH THEO NGUYÊN LÝ THIẾT KẾ:
+Phân tích theo nguyên lý thiết kế: Một agent thực thụ đòi hỏi chu trình ReAct (Reasoning + Acting) khép kín: Suy nghĩ (Thought) -&gt; Hành động gọi tool (Action) -&gt; Quan sát kết quả từ môi trường (Observation) -&gt; Phản hồi. Hệ thống trong đề bài chỉ là luồng đường ống một chiều (static pipeline) nhúng thông tin có sẵn vào prompt trước khi gọi mô hình một lần duy nhất, không có vòng lặp hành vi tự thích ứng.
+NGUỒN THAM KHẢO &amp; TÀI LIỆU KỸ THUẬT:
+Yao, S., et al. (2022). ReAct: Synergizing Reasoning and Acting in Language Models. arXiv:2210.03629. https://arxiv.org/abs/2210.03629; LangChain Documentation - Agent Concepts (https://python.langchain.com/docs/concepts/agents/)</t>
         </is>
       </c>
     </row>
@@ -1412,10 +1424,18 @@
       <c r="K19" s="3" t="inlineStr">
         <is>
           <t>👉 Tiêu chí chấm (Rubric 3 điểm):
-- Đúng bản chất vấn đề và yêu cầu kỹ thuật.
-- Đầy đủ các tiêu chí chấp nhận / test case tối thiểu.
-- Gợi ý cốt lõi: Nhân số token của mỗi chuỗi với số lần lặp; đừng dùng số từ.
-Phân tích theo nguyên lý thiết kế: Nhân số token của mỗi chuỗi với số lần lặp; đừng dùng số từ.</t>
+- Giải thích bản chất Tokenizer (1.5 điểm): Nêu rõ cơ chế sub-word tokenization (BPE/WordPiece) phụ thuộc vào tần suất từ vựng khiến cùng số từ nhưng khác số token.
+- Tính toán và kết luận chính xác (1.5 điểm): Tính đúng A = 7.000 token, B = 13.000 token và khẳng định Chuỗi B tốn ngữ cảnh hơn chuỗi A 6.000 token.
+CÂU TRẢ LỜI MẪU CHI TIẾT:
+1. Giải thích vì sao không thể chỉ đếm từ: Các mô hình ngôn ngữ lớn (LLM) không xử lý văn bản theo từng từ nguyên vẹn mà sử dụng các thuật toán token hóa sub-word (như BPE, WordPiece, Unigram). Thuật toán này băm văn bản dựa trên tần suất xuất hiện trong tập huấn luyện. Những từ hiếm, từ ghép phức tạp, từ đa âm tiết, ký tự có dấu hoặc thuật ngữ chuyên ngành sẽ bị chia tách thành nhiều sub-tokens hoặc các byte đơn lẻ. Do đó, hai chuỗi có cùng số từ (5 từ) nhưng có thể chênh lệch rất lớn về số lượng token thực tế tùy thuộc vào độ quen thuộc của từ vựng.
+2. So sánh lượng ngữ cảnh tiêu tốn:
+- Chuỗi A khi lặp 1.000 lần: 7 token × 1.000 = 7.000 token.
+- Chuỗi B khi lặp 1.000 lần: 13 token × 1.000 = 13.000 token.
+Kết luận: Chuỗi B tốn ngữ cảnh hơn chuỗi A nhiều lần (13.000 token so với 7.000 token, chênh lệch 6.000 token, tốn gấp ~1,86 lần).
+PHÂN TÍCH THEO NGUYÊN LÝ THIẾT KẾ:
+Phân tích theo nguyên lý thiết kế: Cửa sổ ngữ cảnh (context window), thông lượng (throughput) và chi phí API đều được định lượng theo đơn vị Token. Việc ước tính tài nguyên theo số từ (word count) là sai lầm phổ biến dẫn đến lỗi tràn ngữ cảnh (context overflow) hoặc vượt ngân sách chi phí khi xử lý các ngôn ngữ có hình thái phong phú hoặc dữ liệu phi tiếng Anh.
+NGUỒN THAM KHẢO &amp; TÀI LIỆU KỸ THUẬT:
+OpenAI Documentation - What are tokens and how to count them? https://platform.openai.com/docs/guides/embeddings; Sennrich, R., et al. (2016). Neural Machine Translation of Rare Words with Subword Units. https://arxiv.org/abs/1508.07909</t>
         </is>
       </c>
     </row>

</xml_diff>